<commit_message>
Update script mobile ppa Team
</commit_message>
<xml_diff>
--- a/DataDriven/SOS.xlsx
+++ b/DataDriven/SOS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/VScode/QA PPA Team (Android)/DataDriven/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aldopriamnistikogmail.com/Projects/Project_Automation_RobotFramework_StarAsiaPerkasa/DataDriven/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53C536EB-FE7D-6647-90EA-B55E24695B0C}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB4CC311-3111-7B41-8103-5788F3035265}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2780" yWindow="1500" windowWidth="28040" windowHeight="17440" xr2:uid="{1687D09C-A1BE-DC46-9471-D4F815E1B23B}"/>
+    <workbookView xWindow="1360" yWindow="660" windowWidth="28040" windowHeight="17180" xr2:uid="{1687D09C-A1BE-DC46-9471-D4F815E1B23B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>